<commit_message>
BDOI-format FRS of Cashiering v3.2, Product Maintenance v1.2 and User Access Maintenance v1.3 with every screenshot captured again on the corrected platform (walkthroughs included), the workbooks and highlighted copies rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_RTM_BRD-03_Test_Cases_and_Traceability_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_RTM_BRD-03_Test_Cases_and_Traceability_v1.0.xlsx
@@ -3659,7 +3659,7 @@
       </c>
       <c r="H32" s="12" t="inlineStr">
         <is>
-          <t>WT-A.15, WT-A.16, WT-A.17, WT-A.20, WT-B.10 ..., WT-B.9</t>
+          <t>WT-A.14, WT-A.15, WT-A.16, WT-A.17, WT-A.20, WT-B.10 ..., WT-B.9, WT-B.9 ...</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="H68" s="12" t="inlineStr">
         <is>
-          <t>WT-A.12, WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1, WT-B.1 ..., WT-B.2, WT-B.3, WT-B.4 ...</t>
+          <t>WT-A.12, WT-A.14, WT-A.14 ..., WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1, WT-B.2, WT-B.3 ...</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="H77" s="12" t="inlineStr">
         <is>
-          <t>WT-A.10, WT-A.13, WT-A.14 ..., WT-A.7, WT-A.8, WT-A.9, WT-B.5, WT-B.6</t>
+          <t>WT-A.10, WT-A.13, WT-A.7, WT-A.8, WT-A.9, WT-B.5, WT-B.5 ..., WT-B.6</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="H78" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -5691,7 +5691,7 @@
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>WT-A.12, WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1, WT-B.1 ..., WT-B.2</t>
+          <t>WT-A.12, WT-A.14 ..., WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1, WT-B.2</t>
         </is>
       </c>
     </row>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>WT-A.10, WT-A.13, WT-A.14 ..., WT-A.7, WT-A.8, WT-A.9</t>
+          <t>WT-A.10, WT-A.13, WT-A.7, WT-A.8, WT-A.9, WT-B.5 ...</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="H92" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="H98" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="H105" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="H107" s="12" t="inlineStr">
         <is>
-          <t>WT-A.12, WT-A.15, WT-A.16, WT-A.16 ..., WT-A.17, WT-A.20, WT-A.4, WT-A.5, WT-A.6, WT-B.10 ..., WT-B.9</t>
+          <t>WT-A.12, WT-A.14, WT-A.15, WT-A.15 ..., WT-A.16, WT-A.17, WT-A.20, WT-A.4, WT-A.5, WT-A.6, WT-B.9 ...</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
       </c>
       <c r="H108" s="12" t="inlineStr">
         <is>
-          <t>WT-A.15, WT-A.16, WT-A.17, WT-A.20, WT-B.10 ..., WT-B.9</t>
+          <t>WT-A.14, WT-A.15, WT-A.16, WT-A.17, WT-A.20, WT-B.10 ..., WT-B.9, WT-B.9 ...</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="H110" s="12" t="inlineStr">
         <is>
-          <t>WT-A.12, WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1 ...</t>
+          <t>WT-A.12, WT-A.14 ..., WT-A.3, WT-A.4, WT-A.5, WT-A.6</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="H129" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -8331,7 +8331,7 @@
       </c>
       <c r="H149" s="12" t="inlineStr">
         <is>
-          <t>WT-A.12, WT-A.3, WT-A.4, WT-A.5, WT-A.6, WT-B.1 ...</t>
+          <t>WT-A.12, WT-A.14 ..., WT-A.3, WT-A.4, WT-A.5, WT-A.6</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8571,7 @@
       </c>
       <c r="H155" s="12" t="inlineStr">
         <is>
-          <t>WT-A.10, WT-A.13, WT-A.14 ..., WT-A.7, WT-A.8, WT-A.9</t>
+          <t>WT-A.10, WT-A.13, WT-A.7, WT-A.8, WT-A.9, WT-B.5 ...</t>
         </is>
       </c>
     </row>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="H156" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -8691,7 +8691,7 @@
       </c>
       <c r="H158" s="12" t="inlineStr">
         <is>
-          <t>WT-A.13, WT-A.14, WT-B.8</t>
+          <t>WT-A.13, WT-B.8</t>
         </is>
       </c>
     </row>
@@ -31505,7 +31505,7 @@
 MSG-PM-049: "Rates and amounts cannot be negative" (PKG_AMOUNT_NEGATIVE)
 MSG-PM-050: "The insurer chosen did not offer terms in this round" (PKG_INSURER_NOT_OFFERED)
 MSG-PM-051: "Unknown role &lt;given&gt;" (PKG_INSURER_ROLE_INVALID)
-MSG-PM-052: "Enter the rate offered by &lt;insurer name&gt; (&lt;outcome&gt;)" (PKG_RESPONSE_RATE_REQUIRED)
+MSG-PM-052: "Enter the rate offered by &lt;insurer name&gt; (&lt;&gt;)" (PKG_RESPONSE_RATE_REQUIRED)
 MSG-PM-053: "Round &lt;round no&gt; is closed: key in the latest round" (PKG_ROUND_CLOSED)
 MSG-PM-054: "Marketing reviews the terms of a client-specific package" (PKG_SCOPE_CLIENT)
 MSG-PM-055: "A generic programme goes straight to the requirements" (PKG_SCOPE_GENERIC)

</xml_diff>